<commit_message>
GPT-5.5 Pro (웹) Hard 추가
</commit_message>
<xml_diff>
--- a/2026 수능 LLM 풀이 hard.xlsx
+++ b/2026 수능 LLM 풀이 hard.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -710,6 +710,11 @@
           <t>Solar Pro 3 (low)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -838,6 +843,9 @@
       <c r="AP3" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -966,6 +974,9 @@
       <c r="AP4" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -1094,6 +1105,9 @@
       <c r="AP5" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1224,6 +1238,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -1353,6 +1370,9 @@
         <is>
           <t>(포기)</t>
         </is>
+      </c>
+      <c r="AQ7" s="24" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1484,6 +1504,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -1614,6 +1637,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -1744,6 +1770,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -1874,6 +1903,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -2002,6 +2034,9 @@
       <c r="AP12" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -2132,6 +2167,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -2260,6 +2298,9 @@
       <c r="AP14" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -2388,6 +2429,9 @@
       <c r="AP15" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -2516,6 +2560,9 @@
       <c r="AP16" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -2644,6 +2691,9 @@
       <c r="AP17" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -2772,6 +2822,9 @@
       <c r="AP18" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -2900,6 +2953,9 @@
       <c r="AP19" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -3028,6 +3084,9 @@
       <c r="AP20" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -3156,6 +3215,9 @@
       <c r="AP21" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -3284,6 +3346,9 @@
       <c r="AP22" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -3412,6 +3477,9 @@
       <c r="AP23" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ23" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -3540,6 +3608,9 @@
       <c r="AP24" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ24" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -3668,6 +3739,9 @@
       <c r="AP25" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ25" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -3796,6 +3870,9 @@
       <c r="AP26" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ26" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -3924,6 +4001,9 @@
       <c r="AP27" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ27" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -4052,6 +4132,9 @@
       <c r="AP28" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ28" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -4182,6 +4265,9 @@
       <c r="AP29" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ29" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -4312,6 +4398,9 @@
       <c r="AP30" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ30" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -4442,6 +4531,9 @@
       <c r="AP31" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ31" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -4572,6 +4664,9 @@
       <c r="AP32" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ32" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -4702,6 +4797,9 @@
       <c r="AP33" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ33" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -4832,6 +4930,9 @@
       <c r="AP34" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ34" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -4962,6 +5063,9 @@
       <c r="AP35" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ35" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -5092,6 +5196,9 @@
       <c r="AP36" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ36" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -5225,6 +5332,9 @@
       </c>
       <c r="AP38" s="24" t="n">
         <v>56</v>
+      </c>
+      <c r="AQ38" s="24" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="39">
@@ -9089,7 +9199,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -9316,6 +9426,11 @@
           <t>Solar Pro 3 (low)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -9450,6 +9565,9 @@
       <c r="AP3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -9588,6 +9706,9 @@
       <c r="AP4" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -9722,6 +9843,9 @@
       <c r="AP5" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -9862,6 +9986,9 @@
       <c r="AP6" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -10004,6 +10131,9 @@
         <v>4</v>
       </c>
       <c r="AP7" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ7" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10152,6 +10282,9 @@
       <c r="AP8" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -10296,6 +10429,9 @@
       <c r="AP9" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -10440,6 +10576,9 @@
       <c r="AP10" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -10582,6 +10721,9 @@
       <c r="AP11" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -10724,6 +10866,9 @@
       <c r="AP12" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -10868,6 +11013,9 @@
       <c r="AP13" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -11014,6 +11162,9 @@
       <c r="AP14" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -11164,6 +11315,9 @@
       <c r="AP15" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -11312,6 +11466,9 @@
       <c r="AP16" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -11460,6 +11617,9 @@
       <c r="AP17" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -11608,6 +11768,9 @@
       <c r="AP18" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -11756,6 +11919,9 @@
       <c r="AP19" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -11904,6 +12070,9 @@
       <c r="AP20" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -12052,6 +12221,9 @@
       <c r="AP21" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -12200,6 +12372,9 @@
       <c r="AP22" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -12333,6 +12508,9 @@
       </c>
       <c r="AP24" s="24" t="n">
         <v>19</v>
+      </c>
+      <c r="AQ24" s="24" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="25">
@@ -16253,7 +16431,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -16480,6 +16658,11 @@
           <t>Solar Pro 3 (high)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -16622,6 +16805,9 @@
       <c r="AP3" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -16764,6 +16950,9 @@
       <c r="AP4" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -16908,6 +17097,9 @@
       <c r="AP5" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -17052,6 +17244,9 @@
       <c r="AP6" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -17195,6 +17390,9 @@
       </c>
       <c r="AP7" s="25" t="n">
         <v>1</v>
+      </c>
+      <c r="AQ7" s="24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -17342,6 +17540,9 @@
       <c r="AP8" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -17488,6 +17689,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -17636,6 +17840,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -17786,6 +17993,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -17934,6 +18144,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -18086,6 +18299,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -18236,6 +18452,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -18386,6 +18605,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -18536,6 +18758,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -18686,6 +18911,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -18840,6 +19068,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -18992,6 +19223,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -19146,6 +19380,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -19302,6 +19539,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -19456,6 +19696,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -19589,6 +19832,9 @@
       </c>
       <c r="AP24" s="24" t="n">
         <v>9</v>
+      </c>
+      <c r="AQ24" s="24" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="25">
@@ -23509,7 +23755,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -23736,6 +23982,11 @@
           <t>Solar Pro 3 (low)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -23874,6 +24125,9 @@
       <c r="AP3" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -24012,6 +24266,9 @@
       <c r="AP4" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -24150,6 +24407,9 @@
       <c r="AP5" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -24288,6 +24548,9 @@
       <c r="AP6" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -24427,6 +24690,9 @@
         <is>
           <t>(포기)</t>
         </is>
+      </c>
+      <c r="AQ7" s="24" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -24568,6 +24834,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -24706,6 +24975,9 @@
       <c r="AP9" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -24844,6 +25116,9 @@
       <c r="AP10" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -24986,6 +25261,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -25126,6 +25404,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -25268,6 +25549,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -25408,6 +25692,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -25550,6 +25837,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -25694,6 +25984,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -25838,6 +26131,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -25982,6 +26278,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -26126,6 +26425,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -26270,6 +26572,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -26416,6 +26721,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -26560,6 +26868,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -26693,6 +27004,9 @@
       </c>
       <c r="AP24" s="24" t="n">
         <v>7</v>
+      </c>
+      <c r="AQ24" s="24" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="25">
@@ -30613,7 +30927,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -30840,6 +31154,11 @@
           <t>MiniMax M3 (Thinking)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -30970,6 +31289,9 @@
       <c r="AP3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -31102,6 +31424,9 @@
       <c r="AP4" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -31234,6 +31559,9 @@
       <c r="AP5" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -31366,6 +31694,9 @@
       <c r="AP6" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -31496,6 +31827,9 @@
         <v>5</v>
       </c>
       <c r="AP7" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ7" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -31632,6 +31966,9 @@
       <c r="AP8" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -31766,6 +32103,9 @@
       <c r="AP9" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AQ9" s="25" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -31900,6 +32240,9 @@
       <c r="AP10" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AQ10" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -32034,6 +32377,9 @@
       <c r="AP11" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -32170,6 +32516,9 @@
       <c r="AP12" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -32304,6 +32653,9 @@
       <c r="AP13" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -32438,6 +32790,9 @@
       <c r="AP14" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -32574,6 +32929,9 @@
       <c r="AP15" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -32708,6 +33066,9 @@
       <c r="AP16" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -32842,6 +33203,9 @@
       <c r="AP17" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -32976,6 +33340,9 @@
       <c r="AP18" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -33110,6 +33477,9 @@
       <c r="AP19" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -33244,6 +33614,9 @@
       <c r="AP20" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -33378,6 +33751,9 @@
       <c r="AP21" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -33514,6 +33890,9 @@
       <c r="AP22" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -33647,6 +34026,9 @@
       </c>
       <c r="AP24" s="24" t="n">
         <v>36</v>
+      </c>
+      <c r="AQ24" s="24" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="25">
@@ -37567,7 +37949,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -37796,6 +38178,11 @@
           <t>Solar Pro 3 (low)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -37924,6 +38311,9 @@
       <c r="AP3" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -38052,6 +38442,9 @@
       <c r="AP4" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -38182,6 +38575,9 @@
       <c r="AP5" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -38312,6 +38708,9 @@
       <c r="AP6" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -38442,6 +38841,9 @@
       <c r="AP7" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ7" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -38572,6 +38974,9 @@
       <c r="AP8" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -38702,6 +39107,9 @@
       <c r="AP9" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -38832,6 +39240,9 @@
       <c r="AP10" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -38962,6 +39373,9 @@
       <c r="AP11" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -39092,6 +39506,9 @@
       <c r="AP12" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -39224,6 +39641,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -39357,6 +39777,9 @@
       </c>
       <c r="AP15" s="24" t="n">
         <v>15</v>
+      </c>
+      <c r="AQ15" s="24" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -43313,7 +43736,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -43544,6 +43967,11 @@
           <t>Solar Pro 3 (high)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -43674,6 +44102,9 @@
       <c r="AP3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -43806,6 +44237,9 @@
       <c r="AP4" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -43940,6 +44374,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -44072,6 +44509,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -44204,6 +44644,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ7" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -44336,6 +44779,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -44470,6 +44916,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -44602,6 +45051,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -44734,6 +45186,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -44866,6 +45321,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -44998,6 +45456,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -45131,6 +45592,9 @@
       </c>
       <c r="AP15" s="24" t="n">
         <v>0</v>
+      </c>
+      <c r="AQ15" s="24" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -49087,7 +49551,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP37"/>
+  <dimension ref="A1:AQ37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -49314,6 +49778,11 @@
           <t>GLM-5.2 (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -49446,6 +49915,9 @@
       <c r="AP3" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -49578,6 +50050,9 @@
       <c r="AP4" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -49710,6 +50185,9 @@
       <c r="AP5" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -49842,6 +50320,9 @@
       <c r="AP6" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -49972,6 +50453,9 @@
         <v>3</v>
       </c>
       <c r="AP7" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AQ7" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -50106,6 +50590,9 @@
       <c r="AP8" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -50238,6 +50725,9 @@
       <c r="AP9" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -50372,6 +50862,9 @@
       <c r="AP10" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -50506,6 +50999,9 @@
       <c r="AP11" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -50646,6 +51142,9 @@
       <c r="AP12" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -50782,6 +51281,9 @@
       <c r="AP13" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -50918,6 +51420,9 @@
       <c r="AP14" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -51054,6 +51559,9 @@
       <c r="AP15" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -51194,6 +51702,9 @@
       <c r="AP16" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -51336,6 +51847,9 @@
       <c r="AP17" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -51472,6 +51986,9 @@
       <c r="AP18" s="26" t="n">
         <v>9</v>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -51608,6 +52125,9 @@
       <c r="AP19" s="26" t="n">
         <v>16</v>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -51748,6 +52268,9 @@
       <c r="AP20" s="26" t="n">
         <v>12</v>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -51888,6 +52411,9 @@
       <c r="AP21" s="26" t="n">
         <v>15</v>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -52036,6 +52562,9 @@
       <c r="AP22" s="25" t="n">
         <v>-18</v>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -52190,6 +52719,9 @@
       <c r="AP23" s="25" t="n">
         <v>-10</v>
       </c>
+      <c r="AQ23" s="24" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -52346,6 +52878,9 @@
       <c r="AP24" s="25" t="n">
         <v>1474</v>
       </c>
+      <c r="AQ24" s="24" t="n">
+        <v>457</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -52479,6 +53014,9 @@
       </c>
       <c r="AP26" s="24" t="n">
         <v>38</v>
+      </c>
+      <c r="AQ26" s="24" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="27">
@@ -52539,7 +53077,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP37"/>
+  <dimension ref="A1:AQ37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -52766,6 +53304,11 @@
           <t>GLM-5.2 (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -52894,6 +53437,9 @@
       <c r="AP3" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -53022,6 +53568,9 @@
       <c r="AP4" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -53152,6 +53701,9 @@
       <c r="AP5" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -53280,6 +53832,9 @@
       <c r="AP6" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -53410,6 +53965,9 @@
       <c r="AP7" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AQ7" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -53548,6 +54106,9 @@
       <c r="AP8" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -53684,6 +54245,9 @@
       <c r="AP9" s="25" t="n">
         <v>457</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>977</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -53824,6 +54388,9 @@
       <c r="AP10" s="25" t="n">
         <v>78</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>262</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -53957,6 +54524,9 @@
       </c>
       <c r="AP12" s="24" t="n">
         <v>12</v>
+      </c>
+      <c r="AQ12" s="24" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -54069,7 +54639,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -54298,6 +54868,11 @@
           <t>Solar Pro 3 (low)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -54430,6 +55005,9 @@
       <c r="AP3" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -54562,6 +55140,9 @@
       <c r="AP4" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -54694,6 +55275,9 @@
       <c r="AP5" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -54826,6 +55410,9 @@
       <c r="AP6" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -54958,6 +55545,9 @@
       <c r="AP7" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ7" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -55090,6 +55680,9 @@
       <c r="AP8" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -55226,6 +55819,9 @@
       <c r="AP9" s="25" t="n">
         <v>43</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>97</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -55372,6 +55968,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -55505,6 +56104,9 @@
       </c>
       <c r="AP12" s="24" t="n">
         <v>18</v>
+      </c>
+      <c r="AQ12" s="24" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -59473,7 +60075,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP37"/>
+  <dimension ref="A1:AQ37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -59700,6 +60302,11 @@
           <t>Solar Pro 3 (low)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -59830,6 +60437,9 @@
       <c r="AP3" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -59960,6 +60570,9 @@
       <c r="AP4" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -60094,6 +60707,9 @@
       <c r="AP5" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -60226,6 +60842,9 @@
       <c r="AP6" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -60358,6 +60977,9 @@
       <c r="AP7" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ7" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -60488,6 +61110,9 @@
       <c r="AP8" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -60622,6 +61247,9 @@
       <c r="AP9" s="25" t="n">
         <v>72</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>360</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -60754,6 +61382,9 @@
       <c r="AP10" s="25" t="n">
         <v>21</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>221</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -60887,6 +61518,9 @@
       </c>
       <c r="AP12" s="24" t="n">
         <v>18</v>
+      </c>
+      <c r="AQ12" s="24" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -60999,7 +61633,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -61229,6 +61863,11 @@
           <t>Solar Pro 3 (high)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -61357,6 +61996,9 @@
       <c r="AP3" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -61485,6 +62127,9 @@
       <c r="AP4" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -61613,6 +62258,9 @@
       <c r="AP5" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -61747,6 +62395,9 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -61873,6 +62524,9 @@
         <v>4</v>
       </c>
       <c r="AP7" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ7" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -62003,6 +62657,9 @@
       <c r="AP8" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -62131,6 +62788,9 @@
       <c r="AP9" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -62259,6 +62919,9 @@
       <c r="AP10" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -62387,6 +63050,9 @@
       <c r="AP11" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -62515,6 +63181,9 @@
       <c r="AP12" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -62643,6 +63312,9 @@
       <c r="AP13" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -62771,6 +63443,9 @@
       <c r="AP14" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -62899,6 +63574,9 @@
       <c r="AP15" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -63027,6 +63705,9 @@
       <c r="AP16" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -63155,6 +63836,9 @@
       <c r="AP17" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -63283,6 +63967,9 @@
       <c r="AP18" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -63411,6 +64098,9 @@
       <c r="AP19" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -63539,6 +64229,9 @@
       <c r="AP20" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -63667,6 +64360,9 @@
       <c r="AP21" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -63795,6 +64491,9 @@
       <c r="AP22" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -63923,6 +64622,9 @@
       <c r="AP23" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ23" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -64051,6 +64753,9 @@
       <c r="AP24" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ24" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -64179,6 +64884,9 @@
       <c r="AP25" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ25" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -64307,6 +65015,9 @@
       <c r="AP26" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ26" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -64439,6 +65150,9 @@
       <c r="AP27" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ27" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -64567,6 +65281,9 @@
       <c r="AP28" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ28" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -64695,6 +65412,9 @@
       <c r="AP29" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ29" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -64823,6 +65543,9 @@
       <c r="AP30" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ30" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -64951,6 +65674,9 @@
       <c r="AP31" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ31" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -65079,6 +65805,9 @@
       <c r="AP32" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ32" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -65209,6 +65938,9 @@
       <c r="AP33" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ33" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -65339,6 +66071,9 @@
       <c r="AP34" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ34" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -65469,6 +66204,9 @@
       <c r="AP35" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ35" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -65599,6 +66337,9 @@
       <c r="AP36" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ36" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -65729,6 +66470,9 @@
       <c r="AP37" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AQ37" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -65859,6 +66603,9 @@
       <c r="AP38" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ38" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -65989,6 +66736,9 @@
       <c r="AP39" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ39" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
@@ -66119,6 +66869,9 @@
       <c r="AP40" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ40" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
@@ -66249,6 +67002,9 @@
       <c r="AP41" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ41" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -66381,6 +67137,9 @@
       <c r="AP42" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ42" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
@@ -66511,6 +67270,9 @@
       <c r="AP43" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ43" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -66641,6 +67403,9 @@
       <c r="AP44" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AQ44" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
@@ -66771,6 +67536,9 @@
       <c r="AP45" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ45" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -66901,6 +67669,9 @@
       <c r="AP46" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ46" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
@@ -67031,6 +67802,9 @@
       <c r="AP47" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ47" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -67164,6 +67938,9 @@
       </c>
       <c r="AP49" s="24" t="n">
         <v>82</v>
+      </c>
+      <c r="AQ49" s="24" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="50">
@@ -70984,7 +71761,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP1000"/>
+  <dimension ref="A1:AQ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -71215,6 +71992,11 @@
           <t>Solar Pro 3 (low)</t>
         </is>
       </c>
+      <c r="AQ2" s="23" t="inlineStr">
+        <is>
+          <t>GPT-5.5 Pro</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -71343,6 +72125,9 @@
       <c r="AP3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -71471,6 +72256,9 @@
       <c r="AP4" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AQ4" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -71599,6 +72387,9 @@
       <c r="AP5" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AQ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -71727,6 +72518,9 @@
       <c r="AP6" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -71854,6 +72648,9 @@
       </c>
       <c r="AP7" s="25" t="n">
         <v>5</v>
+      </c>
+      <c r="AQ7" s="24" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -71983,6 +72780,9 @@
       <c r="AP8" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -72111,6 +72911,9 @@
       <c r="AP9" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -72239,6 +73042,9 @@
       <c r="AP10" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -72367,6 +73173,9 @@
       <c r="AP11" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -72495,6 +73304,9 @@
       <c r="AP12" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ12" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -72623,6 +73435,9 @@
       <c r="AP13" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -72751,6 +73566,9 @@
       <c r="AP14" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -72879,6 +73697,9 @@
       <c r="AP15" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ15" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -73007,6 +73828,9 @@
       <c r="AP16" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ16" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -73135,6 +73959,9 @@
       <c r="AP17" s="26" t="n">
         <v>3</v>
       </c>
+      <c r="AQ17" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -73263,6 +74090,9 @@
       <c r="AP18" s="26" t="n">
         <v>5</v>
       </c>
+      <c r="AQ18" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -73391,6 +74221,9 @@
       <c r="AP19" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ19" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -73519,6 +74352,9 @@
       <c r="AP20" s="26" t="n">
         <v>2</v>
       </c>
+      <c r="AQ20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -73647,6 +74483,9 @@
       <c r="AP21" s="26" t="n">
         <v>1</v>
       </c>
+      <c r="AQ21" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -73775,6 +74614,9 @@
       <c r="AP22" s="26" t="n">
         <v>4</v>
       </c>
+      <c r="AQ22" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -73908,6 +74750,9 @@
       </c>
       <c r="AP24" s="24" t="n">
         <v>40</v>
+      </c>
+      <c r="AQ24" s="24" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Kimi K2.6, Gemini 2.5 Pro hard 추가
</commit_message>
<xml_diff>
--- a/2026 수능 LLM 풀이 hard.xlsx
+++ b/2026 수능 LLM 풀이 hard.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -745,6 +745,21 @@
           <t>Qwen3.6 27B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -894,6 +909,15 @@
       <c r="AW3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -1043,6 +1067,15 @@
       <c r="AW4" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -1192,6 +1225,15 @@
       <c r="AW5" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1343,6 +1385,15 @@
       <c r="AW6" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -1492,6 +1543,15 @@
         <v>4</v>
       </c>
       <c r="AW7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1645,6 +1705,15 @@
       <c r="AW8" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -1796,6 +1865,15 @@
       <c r="AW9" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX9" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -1947,6 +2025,15 @@
       <c r="AW10" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -2098,6 +2185,15 @@
       <c r="AW11" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -2247,6 +2343,15 @@
       <c r="AW12" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -2398,6 +2503,15 @@
       <c r="AW13" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -2547,6 +2661,15 @@
       <c r="AW14" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ14" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -2696,6 +2819,15 @@
       <c r="AW15" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX15" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -2847,6 +2979,15 @@
       <c r="AW16" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX16" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY16" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ16" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -2998,6 +3139,15 @@
       <c r="AW17" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX17" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY17" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -3149,6 +3299,15 @@
       <c r="AW18" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ18" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -3300,6 +3459,15 @@
       <c r="AW19" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX19" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY19" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ19" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -3451,6 +3619,15 @@
       <c r="AW20" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX20" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -3602,6 +3779,15 @@
       <c r="AW21" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX21" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY21" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ21" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -3753,6 +3939,15 @@
       <c r="AW22" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX22" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY22" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ22" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -3904,6 +4099,15 @@
       <c r="AW23" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX23" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY23" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ23" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -4055,6 +4259,15 @@
       <c r="AW24" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX24" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY24" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -4206,6 +4419,15 @@
       <c r="AW25" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX25" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY25" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ25" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -4357,6 +4579,15 @@
       <c r="AW26" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX26" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY26" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ26" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -4508,6 +4739,15 @@
       <c r="AW27" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX27" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY27" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ27" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -4659,6 +4899,15 @@
       <c r="AW28" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX28" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY28" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ28" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -4812,6 +5061,15 @@
       <c r="AW29" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX29" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY29" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ29" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -4965,6 +5223,15 @@
       <c r="AW30" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX30" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY30" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ30" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -5118,6 +5385,15 @@
       <c r="AW31" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX31" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY31" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ31" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -5271,6 +5547,15 @@
       <c r="AW32" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX32" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY32" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ32" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -5424,6 +5709,15 @@
       <c r="AW33" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ33" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -5577,6 +5871,15 @@
       <c r="AW34" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX34" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY34" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ34" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -5730,6 +6033,15 @@
       <c r="AW35" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX35" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY35" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ35" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -5883,6 +6195,15 @@
       <c r="AW36" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX36" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY36" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ36" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -6037,6 +6358,15 @@
       </c>
       <c r="AW38" s="24" t="n">
         <v>63</v>
+      </c>
+      <c r="AX38" s="24" t="n">
+        <v>65</v>
+      </c>
+      <c r="AY38" s="24" t="n">
+        <v>74</v>
+      </c>
+      <c r="AZ38" s="24" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="39">
@@ -9901,7 +10231,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -10163,6 +10493,21 @@
           <t>Qwen3.6 27B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -10322,6 +10667,15 @@
       <c r="AW3" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -10481,6 +10835,15 @@
       <c r="AW4" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY4" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -10636,6 +10999,15 @@
       <c r="AW5" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -10797,6 +11169,15 @@
       <c r="AW6" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX6" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY6" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -10961,6 +11342,15 @@
       </c>
       <c r="AW7" s="25" t="n">
         <v>4</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY7" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -11131,6 +11521,15 @@
       <c r="AW8" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY8" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ8" s="25" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -11300,6 +11699,15 @@
       <c r="AW9" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -11467,6 +11875,15 @@
       <c r="AW10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -11632,6 +12049,15 @@
       <c r="AW11" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -11797,6 +12223,15 @@
       <c r="AW12" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX12" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY12" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -11966,6 +12401,15 @@
       <c r="AW13" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX13" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY13" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ13" s="25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -12135,6 +12579,17 @@
       <c r="AW14" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ14" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -12310,6 +12765,17 @@
       <c r="AW15" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX15" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ15" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -12483,6 +12949,17 @@
       <c r="AW16" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX16" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY16" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ16" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -12656,6 +13133,17 @@
       <c r="AW17" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX17" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY17" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ17" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -12827,6 +13315,17 @@
       <c r="AW18" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY18" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ18" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -13000,6 +13499,17 @@
       <c r="AW19" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX19" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY19" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ19" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -13173,6 +13683,17 @@
       <c r="AW20" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX20" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY20" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ20" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -13346,6 +13867,17 @@
       <c r="AW21" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX21" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY21" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ21" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -13519,6 +14051,17 @@
       <c r="AW22" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX22" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY22" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ22" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -13673,6 +14216,15 @@
       </c>
       <c r="AW24" s="24" t="n">
         <v>29</v>
+      </c>
+      <c r="AX24" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="AY24" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="25">
@@ -17593,7 +18145,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -17855,6 +18407,21 @@
           <t>Qwen3.6 27B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -18018,6 +18585,15 @@
       <c r="AW3" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -18181,6 +18757,15 @@
       <c r="AW4" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ4" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -18346,6 +18931,15 @@
       <c r="AW5" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -18511,6 +19105,15 @@
       <c r="AW6" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -18675,6 +19278,15 @@
       </c>
       <c r="AW7" s="24" t="n">
         <v>2</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ7" s="25" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -18843,6 +19455,15 @@
       <c r="AW8" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -19010,6 +19631,15 @@
       <c r="AW9" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -19179,6 +19809,15 @@
       <c r="AW10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -19352,6 +19991,15 @@
       <c r="AW11" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY11" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -19523,6 +20171,15 @@
       <c r="AW12" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ12" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -19698,6 +20355,15 @@
       <c r="AW13" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -19871,6 +20537,15 @@
       <c r="AW14" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -20044,6 +20719,15 @@
       <c r="AW15" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX15" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY15" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -20217,6 +20901,15 @@
       <c r="AW16" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX16" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY16" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ16" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -20390,6 +21083,15 @@
       <c r="AW17" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX17" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY17" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -20567,6 +21269,15 @@
       <c r="AW18" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY18" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ18" s="25" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -20742,6 +21453,15 @@
       <c r="AW19" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX19" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY19" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -20919,6 +21639,15 @@
       <c r="AW20" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX20" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY20" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ20" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -21098,6 +21827,15 @@
       <c r="AW21" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX21" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY21" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ21" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -21275,6 +22013,15 @@
       <c r="AW22" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX22" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY22" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ22" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -21429,6 +22176,15 @@
       </c>
       <c r="AW24" s="24" t="n">
         <v>29</v>
+      </c>
+      <c r="AX24" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="AY24" s="24" t="n">
+        <v>45</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="25">
@@ -25349,7 +26105,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -25611,6 +26367,21 @@
           <t>Qwen3.6 27B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -25770,6 +26541,17 @@
       <c r="AW3" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY3" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -25929,6 +26711,17 @@
       <c r="AW4" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY4" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -26088,6 +26881,17 @@
       <c r="AW5" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY5" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -26247,6 +27051,17 @@
       <c r="AW6" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY6" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -26407,6 +27222,17 @@
       </c>
       <c r="AW7" s="25" t="n">
         <v>2</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY7" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ7" s="24" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -26569,6 +27395,17 @@
       <c r="AW8" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX8" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY8" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ8" s="25" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -26728,6 +27565,17 @@
       <c r="AW9" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY9" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -26889,6 +27737,17 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY10" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -27052,6 +27911,17 @@
       <c r="AW11" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX11" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY11" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ11" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -27213,6 +28083,17 @@
       <c r="AW12" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY12" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ12" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -27376,6 +28257,17 @@
       <c r="AW13" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY13" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ13" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -27537,6 +28429,17 @@
       <c r="AW14" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY14" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -27700,6 +28603,17 @@
       <c r="AW15" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX15" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY15" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ15" s="25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -27865,6 +28779,17 @@
       <c r="AW16" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX16" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY16" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ16" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -28030,6 +28955,17 @@
       <c r="AW17" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX17" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY17" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ17" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -28195,6 +29131,17 @@
       <c r="AW18" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY18" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ18" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -28360,6 +29307,17 @@
       <c r="AW19" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY19" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ19" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -28525,6 +29483,17 @@
       <c r="AW20" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX20" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY20" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ20" s="25" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -28692,6 +29661,17 @@
       <c r="AW21" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX21" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY21" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ21" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -28857,6 +29837,17 @@
       <c r="AW22" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY22" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
+      <c r="AZ22" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -29011,6 +30002,15 @@
       </c>
       <c r="AW24" s="24" t="n">
         <v>22</v>
+      </c>
+      <c r="AX24" s="24" t="n">
+        <v>31</v>
+      </c>
+      <c r="AY24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="25">
@@ -32931,7 +33931,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -33193,6 +34193,21 @@
           <t>Qwen3.6 27B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -33346,6 +34361,15 @@
       <c r="AW3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX3" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY3" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -33501,6 +34525,15 @@
       <c r="AW4" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -33656,6 +34689,15 @@
       <c r="AW5" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -33811,6 +34853,15 @@
       <c r="AW6" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -33964,6 +35015,15 @@
         <v>1</v>
       </c>
       <c r="AW7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -34123,6 +35183,15 @@
       <c r="AW8" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -34280,6 +35349,15 @@
       <c r="AW9" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY9" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -34437,6 +35515,15 @@
       <c r="AW10" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX10" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY10" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ10" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -34596,6 +35683,15 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -34759,6 +35855,15 @@
       <c r="AW12" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -34918,6 +36023,15 @@
       <c r="AW13" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY13" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -35077,6 +36191,15 @@
       <c r="AW14" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY14" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ14" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -35238,6 +36361,15 @@
       <c r="AW15" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -35399,6 +36531,15 @@
       <c r="AW16" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX16" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY16" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -35562,6 +36703,17 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AX17" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY17" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ17" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -35721,6 +36873,17 @@
       <c r="AW18" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY18" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ18" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -35880,6 +37043,17 @@
       <c r="AW19" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX19" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY19" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ19" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -36039,6 +37213,17 @@
       <c r="AW20" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ20" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -36198,6 +37383,17 @@
       <c r="AW21" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX21" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY21" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ21" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -36361,6 +37557,17 @@
       <c r="AW22" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX22" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY22" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ22" s="25" t="inlineStr">
+        <is>
+          <t>(포기)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -36515,6 +37722,15 @@
       </c>
       <c r="AW24" s="24" t="n">
         <v>26</v>
+      </c>
+      <c r="AX24" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="AY24" s="24" t="n">
+        <v>43</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="25">
@@ -40435,7 +41651,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -40699,6 +41915,21 @@
           <t>K-EXAONE 236B A23B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -40848,6 +42079,15 @@
       <c r="AW3" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -40997,6 +42237,15 @@
       <c r="AW4" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -41148,6 +42397,15 @@
       <c r="AW5" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -41299,6 +42557,15 @@
       <c r="AW6" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ6" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -41450,6 +42717,15 @@
       <c r="AW7" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ7" s="25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -41601,6 +42877,15 @@
       <c r="AW8" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -41752,6 +43037,15 @@
       <c r="AW9" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -41903,6 +43197,15 @@
       <c r="AW10" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -42054,6 +43357,15 @@
       <c r="AW11" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -42205,6 +43517,15 @@
       <c r="AW12" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -42358,6 +43679,15 @@
       <c r="AW13" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY13" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -42511,6 +43841,15 @@
         <v>24</v>
       </c>
       <c r="AW15" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX15" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
         <v>20</v>
       </c>
     </row>
@@ -46468,7 +47807,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -46734,6 +48073,21 @@
           <t>K-EXAONE 236B A23B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -46885,6 +48239,15 @@
       <c r="AW3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -47038,6 +48401,15 @@
       <c r="AW4" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY4" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -47193,6 +48565,15 @@
       <c r="AW5" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY5" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ5" s="25" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -47346,6 +48727,15 @@
       <c r="AW6" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -47499,6 +48889,15 @@
       <c r="AW7" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ7" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -47652,6 +49051,15 @@
       <c r="AW8" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ8" s="25" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -47807,6 +49215,15 @@
       <c r="AW9" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -47960,6 +49377,15 @@
       <c r="AW10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -48113,6 +49539,15 @@
       <c r="AW11" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -48266,6 +49701,15 @@
       <c r="AW12" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -48419,6 +49863,15 @@
       <c r="AW13" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -48573,6 +50026,15 @@
       </c>
       <c r="AW15" s="24" t="n">
         <v>9</v>
+      </c>
+      <c r="AX15" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -52529,7 +53991,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW37"/>
+  <dimension ref="A1:AZ37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -52791,6 +54253,21 @@
           <t>Qwen3.6 27B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -52944,6 +54421,15 @@
       <c r="AW3" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -53097,6 +54583,15 @@
       <c r="AW4" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -53250,6 +54745,15 @@
       <c r="AW5" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -53403,6 +54907,15 @@
       <c r="AW6" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -53555,6 +55068,15 @@
       </c>
       <c r="AW7" s="25" t="n">
         <v>4</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -53709,6 +55231,15 @@
       <c r="AW8" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -53862,6 +55393,15 @@
       <c r="AW9" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -54017,6 +55557,15 @@
       <c r="AW10" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -54172,6 +55721,15 @@
       <c r="AW11" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -54333,6 +55891,15 @@
       <c r="AW12" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -54492,6 +56059,15 @@
       <c r="AW13" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -54651,6 +56227,15 @@
       <c r="AW14" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -54810,6 +56395,15 @@
       <c r="AW15" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX15" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -54973,6 +56567,15 @@
       <c r="AW16" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX16" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY16" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -55138,6 +56741,15 @@
       <c r="AW17" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX17" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY17" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ17" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -55297,6 +56909,15 @@
       <c r="AW18" s="24" t="n">
         <v>9</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="AY18" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="AZ18" s="24" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -55456,6 +57077,15 @@
       <c r="AW19" s="24" t="n">
         <v>16</v>
       </c>
+      <c r="AX19" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="AY19" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="AZ19" s="24" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -55619,6 +57249,15 @@
       <c r="AW20" s="24" t="n">
         <v>12</v>
       </c>
+      <c r="AX20" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AY20" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AZ20" s="24" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -55782,6 +57421,15 @@
       <c r="AW21" s="24" t="n">
         <v>15</v>
       </c>
+      <c r="AX21" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="AY21" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="AZ21" s="24" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -55955,6 +57603,15 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AX22" s="24" t="n">
+        <v>130</v>
+      </c>
+      <c r="AY22" s="24" t="n">
+        <v>130</v>
+      </c>
+      <c r="AZ22" s="24" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -56134,6 +57791,15 @@
       <c r="AW23" s="25" t="n">
         <v>60</v>
       </c>
+      <c r="AX23" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="AY23" s="24" t="n">
+        <v>65</v>
+      </c>
+      <c r="AZ23" s="24" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -56313,6 +57979,15 @@
       <c r="AW24" s="25" t="n">
         <v>49</v>
       </c>
+      <c r="AX24" s="24" t="n">
+        <v>457</v>
+      </c>
+      <c r="AY24" s="24" t="n">
+        <v>457</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>457</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -56467,6 +58142,15 @@
       </c>
       <c r="AW26" s="24" t="n">
         <v>51</v>
+      </c>
+      <c r="AX26" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="AY26" s="24" t="n">
+        <v>74</v>
+      </c>
+      <c r="AZ26" s="24" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="27">
@@ -56527,7 +58211,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW37"/>
+  <dimension ref="A1:AZ37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -56789,6 +58473,21 @@
           <t>Qwen3.7 Max (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -56938,6 +58637,15 @@
       <c r="AW3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -57087,6 +58795,15 @@
       <c r="AW4" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -57238,6 +58955,15 @@
       <c r="AW5" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -57387,6 +59113,15 @@
       <c r="AW6" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -57538,6 +59273,15 @@
       <c r="AW7" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -57697,6 +59441,15 @@
       <c r="AW8" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -57854,6 +59607,15 @@
       <c r="AW9" s="24" t="n">
         <v>977</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>977</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>977</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>977</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -58015,6 +59777,15 @@
       <c r="AW10" s="25" t="n">
         <v>56</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>262</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>262</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>262</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -58169,6 +59940,15 @@
       </c>
       <c r="AW12" s="24" t="n">
         <v>22</v>
+      </c>
+      <c r="AX12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -58281,7 +60061,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -58545,6 +60325,21 @@
           <t>K-EXAONE 236B A23B (Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -58698,6 +60493,15 @@
       <c r="AW3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -58851,6 +60655,15 @@
       <c r="AW4" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -59004,6 +60817,15 @@
       <c r="AW5" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -59157,6 +60979,15 @@
       <c r="AW6" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -59310,6 +61141,15 @@
       <c r="AW7" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -59463,6 +61303,15 @@
       <c r="AW8" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -59624,6 +61473,15 @@
       <c r="AW9" s="24" t="n">
         <v>97</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>97</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>97</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>97</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -59795,6 +61653,15 @@
       <c r="AW10" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="AZ10" s="25" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -59948,6 +61815,15 @@
         <v>18</v>
       </c>
       <c r="AW12" s="24" t="n">
+        <v>22</v>
+      </c>
+      <c r="AX12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
         <v>22</v>
       </c>
     </row>
@@ -63917,7 +65793,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW37"/>
+  <dimension ref="A1:AZ37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -64179,6 +66055,21 @@
           <t>K-EXAONE 236B A23B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -64330,6 +66221,15 @@
       <c r="AW3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -64481,6 +66381,15 @@
       <c r="AW4" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -64636,6 +66545,15 @@
       <c r="AW5" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -64789,6 +66707,15 @@
       <c r="AW6" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -64942,6 +66869,15 @@
       <c r="AW7" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -65093,6 +67029,15 @@
       <c r="AW8" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ8" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -65250,6 +67195,15 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>360</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>360</v>
+      </c>
+      <c r="AZ9" s="25" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -65407,6 +67361,15 @@
           <t>(포기)</t>
         </is>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>221</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>221</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>221</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -65561,6 +67524,15 @@
       </c>
       <c r="AW12" s="24" t="n">
         <v>14</v>
+      </c>
+      <c r="AX12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="13">
@@ -65673,7 +67645,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -65938,6 +67910,21 @@
           <t>Qwen3.7 Max (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -66087,6 +68074,15 @@
       <c r="AW3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -66236,6 +68232,15 @@
       <c r="AW4" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -66385,6 +68390,15 @@
       <c r="AW5" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -66540,6 +68554,15 @@
       <c r="AW6" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -66687,6 +68710,15 @@
         <v>1</v>
       </c>
       <c r="AW7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -66838,6 +68870,15 @@
       <c r="AW8" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -66987,6 +69028,15 @@
       <c r="AW9" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -67136,6 +69186,15 @@
       <c r="AW10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -67285,6 +69344,15 @@
       <c r="AW11" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -67434,6 +69502,15 @@
       <c r="AW12" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -67583,6 +69660,15 @@
       <c r="AW13" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY13" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -67732,6 +69818,15 @@
       <c r="AW14" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -67881,6 +69976,15 @@
       <c r="AW15" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -68030,6 +70134,15 @@
       <c r="AW16" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX16" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY16" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ16" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -68179,6 +70292,15 @@
       <c r="AW17" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX17" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY17" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ17" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -68328,6 +70450,15 @@
       <c r="AW18" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY18" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ18" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -68477,6 +70608,15 @@
       <c r="AW19" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX19" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY19" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -68626,6 +70766,15 @@
       <c r="AW20" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -68775,6 +70924,15 @@
       <c r="AW21" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX21" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY21" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ21" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -68924,6 +71082,15 @@
       <c r="AW22" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ22" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -69073,6 +71240,15 @@
       <c r="AW23" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX23" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY23" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ23" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -69222,6 +71398,15 @@
       <c r="AW24" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX24" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY24" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -69371,6 +71556,15 @@
       <c r="AW25" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX25" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY25" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ25" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -69520,6 +71714,15 @@
       <c r="AW26" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ26" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -69673,6 +71876,15 @@
       <c r="AW27" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX27" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY27" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ27" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -69822,6 +72034,15 @@
       <c r="AW28" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX28" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY28" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ28" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -69971,6 +72192,15 @@
       <c r="AW29" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX29" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY29" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ29" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -70120,6 +72350,15 @@
       <c r="AW30" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX30" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY30" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ30" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -70269,6 +72508,15 @@
       <c r="AW31" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ31" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -70418,6 +72666,15 @@
       <c r="AW32" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX32" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY32" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ32" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -70569,6 +72826,15 @@
       <c r="AW33" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX33" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY33" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ33" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -70720,6 +72986,15 @@
       <c r="AW34" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX34" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY34" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ34" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -70871,6 +73146,15 @@
       <c r="AW35" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX35" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY35" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ35" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -71022,6 +73306,15 @@
       <c r="AW36" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX36" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY36" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ36" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -71173,6 +73466,15 @@
       <c r="AW37" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX37" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY37" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ37" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -71324,6 +73626,15 @@
       <c r="AW38" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX38" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY38" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ38" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -71475,6 +73786,15 @@
       <c r="AW39" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX39" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY39" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ39" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
@@ -71626,6 +73946,15 @@
       <c r="AW40" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX40" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY40" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ40" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
@@ -71777,6 +74106,15 @@
       <c r="AW41" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX41" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY41" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ41" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -71930,6 +74268,15 @@
       <c r="AW42" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX42" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY42" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ42" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
@@ -72081,6 +74428,15 @@
       <c r="AW43" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX43" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY43" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ43" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -72232,6 +74588,15 @@
       <c r="AW44" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX44" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY44" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ44" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
@@ -72383,6 +74748,15 @@
       <c r="AW45" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX45" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY45" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ45" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -72534,6 +74908,15 @@
       <c r="AW46" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX46" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY46" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ46" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
@@ -72685,6 +75068,15 @@
       <c r="AW47" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX47" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY47" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ47" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -72839,6 +75231,15 @@
       </c>
       <c r="AW49" s="24" t="n">
         <v>96</v>
+      </c>
+      <c r="AX49" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="AY49" s="24" t="n">
+        <v>92</v>
+      </c>
+      <c r="AZ49" s="24" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="50">
@@ -76659,7 +79060,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW1000"/>
+  <dimension ref="A1:AZ1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -76925,6 +79326,21 @@
           <t>Qwen3.6 27B (Non-Thinking)</t>
         </is>
       </c>
+      <c r="AX2" s="23" t="inlineStr">
+        <is>
+          <t>Gemini 2.5 Pro (32K Thinking)</t>
+        </is>
+      </c>
+      <c r="AY2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Thinking)</t>
+        </is>
+      </c>
+      <c r="AZ2" s="23" t="inlineStr">
+        <is>
+          <t>Kimi K2.6 (Non-Thinking)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -77074,6 +79490,15 @@
       <c r="AW3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -77225,6 +79650,15 @@
       <c r="AW4" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX4" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY4" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ4" s="25" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -77374,6 +79808,15 @@
       <c r="AW5" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="AX5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY5" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -77523,6 +79966,15 @@
       <c r="AW6" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX6" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY6" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -77670,6 +80122,15 @@
         <v>2</v>
       </c>
       <c r="AW7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ7" s="24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -77821,6 +80282,15 @@
       <c r="AW8" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY8" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -77970,6 +80440,15 @@
       <c r="AW9" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -78119,6 +80598,15 @@
       <c r="AW10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY10" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -78268,6 +80756,15 @@
       <c r="AW11" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX11" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY11" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ11" s="25" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -78417,6 +80914,15 @@
       <c r="AW12" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ12" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -78566,6 +81072,15 @@
       <c r="AW13" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -78715,6 +81230,15 @@
       <c r="AW14" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="AX14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY14" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ14" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -78864,6 +81388,15 @@
       <c r="AW15" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="AX15" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY15" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ15" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -79013,6 +81546,15 @@
       <c r="AW16" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX16" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY16" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ16" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -79162,6 +81704,15 @@
       <c r="AW17" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="AX17" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY17" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AZ17" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -79311,6 +81862,15 @@
       <c r="AW18" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="AX18" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY18" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ18" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -79460,6 +82020,15 @@
       <c r="AW19" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="AX19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ19" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -79609,6 +82178,15 @@
       <c r="AW20" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="AX20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ20" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -79758,6 +82336,15 @@
       <c r="AW21" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="AX21" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY21" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ21" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -79909,6 +82496,15 @@
       <c r="AW22" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="AX22" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY22" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AZ22" s="25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -80063,6 +82659,15 @@
       </c>
       <c r="AW24" s="24" t="n">
         <v>31</v>
+      </c>
+      <c r="AX24" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="AY24" s="24" t="n">
+        <v>44</v>
+      </c>
+      <c r="AZ24" s="24" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Claude Fable 5 hard 추가
</commit_message>
<xml_diff>
--- a/2026 수능 LLM 풀이 hard.xlsx
+++ b/2026 수능 LLM 풀이 hard.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -770,6 +770,11 @@
           <t>Claude Sonnet 5</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -934,6 +939,9 @@
       <c r="BB3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -1098,6 +1106,9 @@
       <c r="BB4" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -1262,6 +1273,9 @@
       <c r="BB5" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1428,6 +1442,9 @@
       <c r="BB6" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -1592,6 +1609,9 @@
         <v>4</v>
       </c>
       <c r="BB7" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BC7" s="24" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1760,6 +1780,9 @@
       <c r="BB8" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -1926,6 +1949,9 @@
       <c r="BB9" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -2092,6 +2118,9 @@
       <c r="BB10" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -2258,6 +2287,9 @@
       <c r="BB11" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -2422,6 +2454,9 @@
       <c r="BB12" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -2588,6 +2623,9 @@
       <c r="BB13" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -2752,6 +2790,9 @@
       <c r="BB14" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC14" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -2916,6 +2957,9 @@
       <c r="BB15" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC15" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -3082,6 +3126,9 @@
       <c r="BB16" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC16" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -3248,6 +3295,9 @@
       <c r="BB17" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -3414,6 +3464,9 @@
       <c r="BB18" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC18" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -3580,6 +3633,9 @@
       <c r="BB19" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC19" s="25" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -3746,6 +3802,9 @@
       <c r="BB20" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -3912,6 +3971,9 @@
       <c r="BB21" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC21" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -4078,6 +4140,9 @@
       <c r="BB22" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC22" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -4244,6 +4309,9 @@
       <c r="BB23" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC23" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -4410,6 +4478,9 @@
       <c r="BB24" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC24" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -4576,6 +4647,9 @@
       <c r="BB25" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC25" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -4742,6 +4816,9 @@
       <c r="BB26" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC26" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -4908,6 +4985,9 @@
       <c r="BB27" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC27" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -5074,6 +5154,9 @@
       <c r="BB28" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC28" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -5242,6 +5325,9 @@
       <c r="BB29" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC29" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -5410,6 +5496,9 @@
       <c r="BB30" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC30" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -5578,6 +5667,9 @@
       <c r="BB31" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC31" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -5746,6 +5838,9 @@
       <c r="BB32" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC32" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -5914,6 +6009,9 @@
       <c r="BB33" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC33" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -6082,6 +6180,9 @@
       <c r="BB34" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC34" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -6250,6 +6351,9 @@
       <c r="BB35" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC35" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -6418,6 +6522,9 @@
       <c r="BB36" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC36" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -6587,6 +6694,9 @@
       </c>
       <c r="BB38" s="24" t="n">
         <v>47</v>
+      </c>
+      <c r="BC38" s="24" t="n">
+        <v>73</v>
       </c>
     </row>
     <row r="39">
@@ -10451,7 +10561,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -10738,6 +10848,11 @@
           <t>Claude Sonnet 5</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -10914,6 +11029,9 @@
       <c r="BB3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -11090,6 +11208,9 @@
       <c r="BB4" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -11262,6 +11383,9 @@
       <c r="BB5" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -11440,6 +11564,9 @@
       <c r="BB6" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -11621,6 +11748,9 @@
       </c>
       <c r="BB7" s="25" t="n">
         <v>3</v>
+      </c>
+      <c r="BC7" s="24" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -11808,6 +11938,9 @@
       <c r="BB8" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC8" s="25" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -11994,6 +12127,9 @@
       <c r="BB9" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -12178,6 +12314,9 @@
       <c r="BB10" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -12360,6 +12499,9 @@
       <c r="BB11" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -12542,6 +12684,9 @@
       <c r="BB12" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -12728,6 +12873,9 @@
       <c r="BB13" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -12916,6 +13064,9 @@
       <c r="BB14" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC14" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -13110,6 +13261,9 @@
       <c r="BB15" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC15" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -13302,6 +13456,9 @@
       <c r="BB16" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC16" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -13494,6 +13651,9 @@
       <c r="BB17" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -13684,6 +13844,9 @@
       <c r="BB18" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC18" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -13876,6 +14039,9 @@
       <c r="BB19" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -14068,6 +14234,9 @@
       <c r="BB20" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -14260,6 +14429,9 @@
       <c r="BB21" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC21" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -14452,6 +14624,9 @@
       <c r="BB22" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC22" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -14621,6 +14796,9 @@
       </c>
       <c r="BB24" s="24" t="n">
         <v>11</v>
+      </c>
+      <c r="BC24" s="24" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="25">
@@ -18541,7 +18719,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -18828,6 +19006,11 @@
           <t>Claude Sonnet 5 (high)</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -19008,6 +19191,9 @@
       <c r="BB3" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -19188,6 +19374,9 @@
       <c r="BB4" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -19370,6 +19559,9 @@
       <c r="BB5" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -19552,6 +19744,9 @@
       <c r="BB6" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -19732,6 +19927,9 @@
         <v>2</v>
       </c>
       <c r="BB7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC7" s="24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -19918,6 +20116,9 @@
       <c r="BB8" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -20102,6 +20303,9 @@
       <c r="BB9" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -20288,6 +20492,9 @@
       <c r="BB10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -20478,6 +20685,9 @@
       <c r="BB11" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -20666,6 +20876,9 @@
       <c r="BB12" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -20858,6 +21071,9 @@
       <c r="BB13" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -21048,6 +21264,9 @@
       <c r="BB14" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -21238,6 +21457,9 @@
       <c r="BB15" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC15" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -21428,6 +21650,9 @@
       <c r="BB16" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -21618,6 +21843,9 @@
       <c r="BB17" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC17" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -21812,6 +22040,9 @@
       <c r="BB18" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC18" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -22004,6 +22235,9 @@
       <c r="BB19" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -22198,6 +22432,9 @@
       <c r="BB20" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC20" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -22394,6 +22631,9 @@
       <c r="BB21" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC21" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -22588,6 +22828,9 @@
       <c r="BB22" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC22" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -22757,6 +23000,9 @@
       </c>
       <c r="BB24" s="24" t="n">
         <v>45</v>
+      </c>
+      <c r="BC24" s="24" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="25">
@@ -26677,7 +26923,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -26964,6 +27210,11 @@
           <t>Claude Sonnet 5</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -27142,6 +27393,11 @@
       <c r="BB3" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC3" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -27320,6 +27576,11 @@
       <c r="BB4" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC4" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -27498,6 +27759,11 @@
       <c r="BB5" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC5" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -27676,6 +27942,11 @@
       <c r="BB6" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC6" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -27855,6 +28126,11 @@
       </c>
       <c r="BB7" s="25" t="n">
         <v>2</v>
+      </c>
+      <c r="BC7" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -28036,6 +28312,11 @@
       <c r="BB8" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC8" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -28214,6 +28495,11 @@
       <c r="BB9" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC9" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -28394,6 +28680,11 @@
       <c r="BB10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC10" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -28576,6 +28867,11 @@
       <c r="BB11" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC11" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -28756,6 +29052,11 @@
       <c r="BB12" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC12" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -28938,6 +29239,11 @@
       <c r="BB13" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC13" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -29118,6 +29424,11 @@
       <c r="BB14" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC14" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -29300,6 +29611,11 @@
       <c r="BB15" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC15" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -29484,6 +29800,11 @@
       <c r="BB16" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC16" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -29668,6 +29989,11 @@
       <c r="BB17" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC17" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -29852,6 +30178,11 @@
       <c r="BB18" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC18" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -30036,6 +30367,11 @@
       <c r="BB19" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC19" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -30220,6 +30556,11 @@
       <c r="BB20" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC20" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -30406,6 +30747,11 @@
       <c r="BB21" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC21" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -30590,6 +30936,11 @@
       <c r="BB22" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC22" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -30759,6 +31110,9 @@
       </c>
       <c r="BB24" s="24" t="n">
         <v>20</v>
+      </c>
+      <c r="BC24" s="24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -34679,7 +35033,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -34966,6 +35320,11 @@
           <t>Claude Sonnet 5</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="20" t="n">
@@ -35136,6 +35495,11 @@
       <c r="BB3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC3" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="20" t="n">
@@ -35308,6 +35672,11 @@
       <c r="BB4" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC4" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="n">
@@ -35480,6 +35849,11 @@
       <c r="BB5" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC5" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="20" t="n">
@@ -35652,6 +36026,11 @@
       <c r="BB6" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC6" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="n">
@@ -35823,6 +36202,11 @@
       </c>
       <c r="BB7" s="25" t="n">
         <v>3</v>
+      </c>
+      <c r="BC7" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -35998,6 +36382,11 @@
       <c r="BB8" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC8" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="n">
@@ -36172,6 +36561,11 @@
       <c r="BB9" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC9" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="20" t="n">
@@ -36346,6 +36740,11 @@
       <c r="BB10" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC10" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="n">
@@ -36522,6 +36921,11 @@
       <c r="BB11" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC11" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="20" t="n">
@@ -36702,6 +37106,11 @@
       <c r="BB12" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC12" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="20" t="n">
@@ -36878,6 +37287,11 @@
       <c r="BB13" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC13" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="20" t="n">
@@ -37054,6 +37468,11 @@
       <c r="BB14" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC14" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="n">
@@ -37232,6 +37651,11 @@
       <c r="BB15" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC15" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="20" t="n">
@@ -37410,6 +37834,11 @@
       <c r="BB16" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC16" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="20" t="n">
@@ -37592,6 +38021,11 @@
       <c r="BB17" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC17" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="20" t="n">
@@ -37770,6 +38204,11 @@
       <c r="BB18" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC18" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="20" t="n">
@@ -37948,6 +38387,11 @@
       <c r="BB19" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC19" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="n">
@@ -38126,6 +38570,11 @@
       <c r="BB20" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC20" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="20" t="n">
@@ -38304,6 +38753,11 @@
       <c r="BB21" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC21" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="20" t="n">
@@ -38486,6 +38940,11 @@
       <c r="BB22" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC22" s="29" t="inlineStr">
+        <is>
+          <t>(검열)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="20" t="n"/>
@@ -38655,6 +39114,9 @@
       </c>
       <c r="BB24" s="24" t="n">
         <v>21</v>
+      </c>
+      <c r="BC24" s="24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -42575,7 +43037,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -42864,6 +43326,11 @@
           <t>Claude Sonnet 5</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -43028,6 +43495,9 @@
       <c r="BB3" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -43192,6 +43662,9 @@
       <c r="BB4" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -43358,6 +43831,9 @@
       <c r="BB5" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -43524,6 +44000,9 @@
       <c r="BB6" s="25" t="n">
         <v>3</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -43690,6 +44169,9 @@
       <c r="BB7" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC7" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -43856,6 +44338,9 @@
       <c r="BB8" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -44022,6 +44507,9 @@
       <c r="BB9" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -44188,6 +44676,9 @@
       <c r="BB10" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -44354,6 +44845,9 @@
       <c r="BB11" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -44520,6 +45014,9 @@
       <c r="BB12" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -44688,6 +45185,9 @@
       <c r="BB13" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -44857,6 +45357,9 @@
       </c>
       <c r="BB15" s="24" t="n">
         <v>14</v>
+      </c>
+      <c r="BC15" s="24" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -48813,7 +49316,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -49104,6 +49607,11 @@
           <t>Claude Sonnet 5</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -49272,6 +49780,9 @@
       <c r="BB3" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -49442,6 +49953,9 @@
       <c r="BB4" s="25" t="n">
         <v>5</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -49614,6 +50128,9 @@
       <c r="BB5" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -49784,6 +50301,9 @@
       <c r="BB6" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -49954,6 +50474,9 @@
       <c r="BB7" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC7" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -50124,6 +50647,9 @@
       <c r="BB8" s="25" t="n">
         <v>1</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -50296,6 +50822,9 @@
       <c r="BB9" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -50466,6 +50995,9 @@
       <c r="BB10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -50636,6 +51168,9 @@
       <c r="BB11" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -50806,6 +51341,9 @@
       <c r="BB12" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -50976,6 +51514,9 @@
       <c r="BB13" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -51145,6 +51686,9 @@
       </c>
       <c r="BB15" s="24" t="n">
         <v>13</v>
+      </c>
+      <c r="BC15" s="24" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="16">
@@ -55101,7 +55645,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB37"/>
+  <dimension ref="A1:BC37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -55388,6 +55932,11 @@
           <t>Claude Sonnet 5 (high)</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -55556,6 +56105,9 @@
       <c r="BB3" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -55724,6 +56276,9 @@
       <c r="BB4" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -55892,6 +56447,9 @@
       <c r="BB5" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -56060,6 +56618,9 @@
       <c r="BB6" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -56226,6 +56787,9 @@
         <v>3</v>
       </c>
       <c r="BB7" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC7" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -56396,6 +56960,9 @@
       <c r="BB8" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -56564,6 +57131,9 @@
       <c r="BB9" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -56734,6 +57304,9 @@
       <c r="BB10" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -56904,6 +57477,9 @@
       <c r="BB11" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -57080,6 +57656,9 @@
       <c r="BB12" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -57254,6 +57833,9 @@
       <c r="BB13" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -57428,6 +58010,9 @@
       <c r="BB14" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -57602,6 +58187,9 @@
       <c r="BB15" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC15" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -57780,6 +58368,9 @@
       <c r="BB16" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC16" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -57960,6 +58551,9 @@
       <c r="BB17" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC17" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -58134,6 +58728,9 @@
       <c r="BB18" s="24" t="n">
         <v>9</v>
       </c>
+      <c r="BC18" s="24" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -58308,6 +58905,9 @@
       <c r="BB19" s="24" t="n">
         <v>16</v>
       </c>
+      <c r="BC19" s="24" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -58486,6 +59086,9 @@
       <c r="BB20" s="24" t="n">
         <v>12</v>
       </c>
+      <c r="BC20" s="24" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -58664,6 +59267,9 @@
       <c r="BB21" s="24" t="n">
         <v>15</v>
       </c>
+      <c r="BC21" s="24" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -58852,6 +59458,9 @@
       <c r="BB22" s="24" t="n">
         <v>130</v>
       </c>
+      <c r="BC22" s="24" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -59046,6 +59655,9 @@
       <c r="BB23" s="24" t="n">
         <v>65</v>
       </c>
+      <c r="BC23" s="24" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -59240,6 +59852,9 @@
       <c r="BB24" s="24" t="n">
         <v>457</v>
       </c>
+      <c r="BC24" s="24" t="n">
+        <v>457</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -59408,6 +60023,9 @@
         <v>50</v>
       </c>
       <c r="BB26" s="24" t="n">
+        <v>74</v>
+      </c>
+      <c r="BC26" s="24" t="n">
         <v>74</v>
       </c>
     </row>
@@ -59469,7 +60087,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB37"/>
+  <dimension ref="A1:BC37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -59756,6 +60374,11 @@
           <t>Claude Sonnet 5 (high)</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -59920,6 +60543,9 @@
       <c r="BB3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -60084,6 +60710,9 @@
       <c r="BB4" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -60250,6 +60879,9 @@
       <c r="BB5" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -60414,6 +61046,9 @@
       <c r="BB6" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -60580,6 +61215,9 @@
       <c r="BB7" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC7" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -60754,6 +61392,9 @@
       <c r="BB8" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -60926,6 +61567,9 @@
       <c r="BB9" s="24" t="n">
         <v>977</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>977</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -61102,6 +61746,9 @@
       <c r="BB10" s="24" t="n">
         <v>262</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>262</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -61270,6 +61917,9 @@
         <v>18</v>
       </c>
       <c r="BB12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="BC12" s="24" t="n">
         <v>26</v>
       </c>
     </row>
@@ -61383,7 +62033,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -61672,6 +62322,11 @@
           <t>Claude Sonnet 5 (high)</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -61840,6 +62495,9 @@
       <c r="BB3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -62008,6 +62666,9 @@
       <c r="BB4" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -62176,6 +62837,9 @@
       <c r="BB5" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -62344,6 +63008,9 @@
       <c r="BB6" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -62512,6 +63179,9 @@
       <c r="BB7" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC7" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -62680,6 +63350,9 @@
       <c r="BB8" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -62856,6 +63529,9 @@
       <c r="BB9" s="24" t="n">
         <v>97</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>97</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -63042,6 +63718,9 @@
       <c r="BB10" s="24" t="n">
         <v>11</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -63210,6 +63889,9 @@
         <v>18</v>
       </c>
       <c r="BB12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="BC12" s="24" t="n">
         <v>26</v>
       </c>
     </row>
@@ -67179,7 +67861,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB37"/>
+  <dimension ref="A1:BC37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -67466,6 +68148,11 @@
           <t>Claude Sonnet 5 (high)</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -67632,6 +68319,9 @@
       <c r="BB3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -67798,6 +68488,9 @@
       <c r="BB4" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -67968,6 +68661,9 @@
       <c r="BB5" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -68136,6 +68832,9 @@
       <c r="BB6" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -68304,6 +69003,9 @@
       <c r="BB7" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC7" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -68470,6 +69172,9 @@
       <c r="BB8" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -68642,6 +69347,9 @@
       <c r="BB9" s="24" t="n">
         <v>360</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>360</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -68814,6 +69522,9 @@
       <c r="BB10" s="24" t="n">
         <v>221</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>221</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -68982,6 +69693,9 @@
         <v>14</v>
       </c>
       <c r="BB12" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="BC12" s="24" t="n">
         <v>26</v>
       </c>
     </row>
@@ -69095,7 +69809,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -69385,6 +70099,11 @@
           <t>Claude Sonnet 5 (high)</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -69549,6 +70268,9 @@
       <c r="BB3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -69713,6 +70435,9 @@
       <c r="BB4" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -69877,6 +70602,9 @@
       <c r="BB5" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -70047,6 +70775,9 @@
       <c r="BB6" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -70209,6 +70940,9 @@
         <v>1</v>
       </c>
       <c r="BB7" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC7" s="24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -70375,6 +71109,9 @@
       <c r="BB8" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -70539,6 +71276,9 @@
       <c r="BB9" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -70703,6 +71443,9 @@
       <c r="BB10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -70867,6 +71610,9 @@
       <c r="BB11" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -71031,6 +71777,9 @@
       <c r="BB12" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -71195,6 +71944,9 @@
       <c r="BB13" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -71359,6 +72111,9 @@
       <c r="BB14" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -71523,6 +72278,9 @@
       <c r="BB15" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC15" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -71687,6 +72445,9 @@
       <c r="BB16" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC16" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -71851,6 +72612,9 @@
       <c r="BB17" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC17" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -72015,6 +72779,9 @@
       <c r="BB18" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC18" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -72179,6 +72946,9 @@
       <c r="BB19" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC19" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -72343,6 +73113,9 @@
       <c r="BB20" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -72507,6 +73280,9 @@
       <c r="BB21" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC21" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -72671,6 +73447,9 @@
       <c r="BB22" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC22" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -72835,6 +73614,9 @@
       <c r="BB23" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC23" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -72999,6 +73781,9 @@
       <c r="BB24" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC24" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -73163,6 +73948,9 @@
       <c r="BB25" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC25" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -73327,6 +74115,9 @@
       <c r="BB26" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC26" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -73495,6 +74286,9 @@
       <c r="BB27" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC27" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -73659,6 +74453,9 @@
       <c r="BB28" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC28" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -73823,6 +74620,9 @@
       <c r="BB29" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC29" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -73987,6 +74787,9 @@
       <c r="BB30" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC30" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -74151,6 +74954,9 @@
       <c r="BB31" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC31" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -74315,6 +75121,9 @@
       <c r="BB32" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC32" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -74481,6 +75290,9 @@
       <c r="BB33" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC33" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -74647,6 +75459,9 @@
       <c r="BB34" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC34" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -74813,6 +75628,9 @@
       <c r="BB35" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC35" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -74979,6 +75797,9 @@
       <c r="BB36" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC36" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -75145,6 +75966,9 @@
       <c r="BB37" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC37" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -75311,6 +76135,9 @@
       <c r="BB38" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC38" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -75477,6 +76304,9 @@
       <c r="BB39" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC39" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
@@ -75643,6 +76473,9 @@
       <c r="BB40" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC40" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
@@ -75809,6 +76642,9 @@
       <c r="BB41" s="25" t="n">
         <v>2</v>
       </c>
+      <c r="BC41" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
@@ -75977,6 +76813,9 @@
       <c r="BB42" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC42" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
@@ -76143,6 +76982,9 @@
       <c r="BB43" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC43" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
@@ -76309,6 +77151,9 @@
       <c r="BB44" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC44" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
@@ -76475,6 +77320,9 @@
       <c r="BB45" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC45" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
@@ -76641,6 +77489,9 @@
       <c r="BB46" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC46" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
@@ -76807,6 +77658,9 @@
       <c r="BB47" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC47" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -76976,6 +77830,9 @@
       </c>
       <c r="BB49" s="24" t="n">
         <v>94</v>
+      </c>
+      <c r="BC49" s="24" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="50">
@@ -80796,7 +81653,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB1000"/>
+  <dimension ref="A1:BC1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="9.5" customWidth="1" style="22" min="1" max="1"/>
@@ -81087,6 +81944,11 @@
           <t>Claude Sonnet 5</t>
         </is>
       </c>
+      <c r="BC2" s="23" t="inlineStr">
+        <is>
+          <t>Claude Fable 5 (high)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n">
@@ -81251,6 +82113,9 @@
       <c r="BB3" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC3" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n">
@@ -81417,6 +82282,9 @@
       <c r="BB4" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC4" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -81581,6 +82449,9 @@
       <c r="BB5" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC5" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -81745,6 +82616,9 @@
       <c r="BB6" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC6" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -81907,6 +82781,9 @@
         <v>2</v>
       </c>
       <c r="BB7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC7" s="24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -82073,6 +82950,9 @@
       <c r="BB8" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC8" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -82237,6 +83117,9 @@
       <c r="BB9" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC9" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -82401,6 +83284,9 @@
       <c r="BB10" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC10" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -82565,6 +83451,9 @@
       <c r="BB11" s="25" t="n">
         <v>4</v>
       </c>
+      <c r="BC11" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -82729,6 +83618,9 @@
       <c r="BB12" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC12" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -82893,6 +83785,9 @@
       <c r="BB13" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC13" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -83057,6 +83952,9 @@
       <c r="BB14" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC14" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -83221,6 +84119,9 @@
       <c r="BB15" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC15" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -83385,6 +84286,9 @@
       <c r="BB16" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC16" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -83549,6 +84453,9 @@
       <c r="BB17" s="24" t="n">
         <v>3</v>
       </c>
+      <c r="BC17" s="24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -83713,6 +84620,9 @@
       <c r="BB18" s="24" t="n">
         <v>5</v>
       </c>
+      <c r="BC18" s="24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -83877,6 +84787,9 @@
       <c r="BB19" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC19" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -84041,6 +84954,9 @@
       <c r="BB20" s="24" t="n">
         <v>2</v>
       </c>
+      <c r="BC20" s="24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -84205,6 +85121,9 @@
       <c r="BB21" s="24" t="n">
         <v>1</v>
       </c>
+      <c r="BC21" s="24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -84371,6 +85290,9 @@
       <c r="BB22" s="24" t="n">
         <v>4</v>
       </c>
+      <c r="BC22" s="24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -84540,6 +85462,9 @@
       </c>
       <c r="BB24" s="24" t="n">
         <v>47</v>
+      </c>
+      <c r="BC24" s="24" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="25">

</xml_diff>